<commit_message>
Update catchment to 25 mi / 1-hr local rules and blank intake template.
Wire staging_radius_miles, drive_minutes, and remote_max_tpd so Local is inclusive of distance or drive-time proxy (40 mph); promote far ≥1.2 tpd sites to Staffed; Remote only when far and below that floor. Document that Lat/Lon + Excel/JSON all live in the Python engine (no geo GUI).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/engine/sample/intake_template.xlsx
+++ b/engine/sample/intake_template.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -454,57 +454,88 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1. Fill the Sites tab. TicketsYr and/or Users/Seats and/or Devices are all accepted.</t>
+          <t>1. Fill the Sites tab (headers only — add one row per site).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2. Leave DepotHub blank to default one virtual campus per Country.</t>
+          <t>2. Geocode addresses externally; put Latitude / Longitude on each site row.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>3. Tweak Settings (yellow conceptually — all Value cells are inputs).</t>
+          <t>3. Leave DepotHub blank to default one virtual campus per Country.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>4. Optional CountryPolicy for customs/language/partner notes.</t>
+          <t>4. Tweak Settings as needed (catchment: staging_radius_miles, drive_minutes, remote_max_tpd).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>5. Run:  python -m engine run path/to/this.xlsx -o Deal_Output.xlsx</t>
+          <t>5. Optional CountryPolicy for customs/language/partner notes.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>6. Run:  python -m engine run path/to/this.xlsx -o Deal_Output.xlsx [--json summary.json]</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Demand resolution order: tickets → users/seats × rate → devices × rate → placeholder (flagged).</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Site columns: Site, Country, Region, City, State, Address, PostalCode, Latitude, Longitude, TicketsYr, Users, Seats, Devices, DepotHub, Customs, CustomerStaffed, CoverageClass, Critical24x7, SpaceNeeded, Zone, Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Demand resolution order: tickets → users/seats × rate → devices × rate → placeholder (flagged).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Catchment: Local if ≤25 mi OR ≤~60 drive-min (40 mph proxy); Remote only if &lt;1.2 tpd and far;</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>far sites with ≥1.2 tpd promote to Staffed campus. No separate geo GUI — Lat/Lon in Excel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
           <t>Sites without coordinates are never auto-classified Local/Staffed by distance.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>No customer names belong in this template — use generic site labels.</t>
         </is>
@@ -521,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -654,336 +685,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Site Alpha HQ</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>NAM</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Austin</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="n">
-        <v>30.27</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-97.73999999999999</v>
-      </c>
-      <c r="J2" t="n">
-        <v>4200</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1800</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>USA-Central</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>Campus</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Site Alpha East</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>NAM</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Dallas</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
-        <v>32.78</v>
-      </c>
-      <c r="I3" t="n">
-        <v>-96.8</v>
-      </c>
-      <c r="J3" t="n">
-        <v>900</v>
-      </c>
-      <c r="K3" t="n">
-        <v>400</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>USA-Central</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>Metro</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Site Beta Hub</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>EMEA</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Frankfurt</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="n">
-        <v>50.11</v>
-      </c>
-      <c r="I4" t="n">
-        <v>8.68</v>
-      </c>
-      <c r="J4" t="n">
-        <v>3100</v>
-      </c>
-      <c r="K4" t="n">
-        <v>1200</v>
-      </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>Campus</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Site Beta Spoke</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Germany</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>EMEA</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Mainz</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="n">
-        <v>49.99</v>
-      </c>
-      <c r="I5" t="n">
-        <v>8.27</v>
-      </c>
-      <c r="J5" t="n">
-        <v>180</v>
-      </c>
-      <c r="K5" t="n">
-        <v>80</v>
-      </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Site Gamma Remote</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>LATAM</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Manaus</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="n">
-        <v>60</v>
-      </c>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Dispatch</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>Remote</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>No coords — remote/uncertain</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Site Delta Devices Only</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>APJC</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Singapore</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="n">
-        <v>1.29</v>
-      </c>
-      <c r="I7" t="n">
-        <v>103.85</v>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="n">
-        <v>500</v>
-      </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>Demand from devices</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -995,12 +696,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C72"/>
+  <dimension ref="A1:C112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1038,15 +739,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>drive_radius_km</t>
+          <t>staging_radius_miles</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Local/Staffed catchment radius</t>
+          <t>Local if haversine miles ≤ this (OR drive-time proxy)</t>
         </is>
       </c>
     </row>
@@ -1059,315 +760,331 @@
       <c r="B4" t="n">
         <v>60</v>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Local if estimated drive minutes ≤ this (at avg_drive_speed_mph)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>incident_share</t>
+          <t>avg_drive_speed_mph</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5</v>
+        <v>40</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0-1; calibrate from ticket extract when available</t>
+          <t>Speed for drive-time proxy; 40 mph → ~40 mi for 60 min</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>onsite_incident_rate</t>
+          <t>remote_max_tpd</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
-      </c>
-      <c r="C6" t="inlineStr"/>
+        <v>1.2</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Remote+dispatch only below this tpd AND outside local range</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>onsite_request_rate</t>
+          <t>drive_radius_km</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
-      </c>
-      <c r="C7" t="inlineStr"/>
+        <v>60</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Legacy — unused; catchment uses miles + drive_minutes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>remote_rate</t>
+          <t>incident_share</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>5</v>
-      </c>
-      <c r="C8" t="inlineStr"/>
+        <v>0.5</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0-1; calibrate from ticket extract when available</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>utilization</t>
+          <t>onsite_incident_rate</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.85</v>
+        <v>6</v>
       </c>
       <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>team_floor</t>
+          <t>onsite_request_rate</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Minimum techs per VC for resilience</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>single_tech_threshold</t>
+          <t>remote_rate</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Tickets/day below which 1-tech exception allowed</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>promotion_threshold_tpd</t>
+          <t>utilization</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4.5</v>
+        <v>0.85</v>
       </c>
       <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>hub_workload_threshold</t>
+          <t>team_floor</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C13" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Minimum techs per VC for resilience</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>lead_span</t>
+          <t>single_tech_threshold</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>10</v>
-      </c>
-      <c r="C14" t="inlineStr"/>
+        <v>2.5</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Tickets/day below which 1-tech team exception allowed (sizing only)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>mgr_span</t>
+          <t>hub_workload_threshold</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>24</v>
+        <v>0.5</v>
       </c>
       <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>estate_tickets_per_user</t>
+          <t>lead_span</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Used when tickets missing but users/seats present</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>estate_tickets_per_device</t>
+          <t>mgr_span</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Used when only device counts present</t>
-        </is>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>placeholder_tickets_per_site</t>
+          <t>estate_tickets_per_user</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>12</v>
+        <v>1.6</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Last-resort demand when no volume fields</t>
+          <t>Used when tickets missing but users/seats present</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>include_cost</t>
+          <t>estate_tickets_per_device</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1 = include labor/cost tabs</t>
+          <t>Used when only device counts present</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>rate_NAM</t>
+          <t>placeholder_tickets_per_site</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>85000</v>
-      </c>
-      <c r="C20" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Last-resort demand when no volume fields</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>rate_LATAM</t>
+          <t>include_cost</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>42000</v>
-      </c>
-      <c r="C21" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1 = include labor/cost tabs</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>rate_EMEA</t>
+          <t>rate_NAM</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>72000</v>
+        <v>85000</v>
       </c>
       <c r="C22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>rate_APJC</t>
+          <t>rate_LATAM</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>40000</v>
+        <v>42000</v>
       </c>
       <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>burden_uplift</t>
+          <t>rate_EMEA</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.28</v>
+        <v>72000</v>
       </c>
       <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>lead_premium</t>
+          <t>rate_APJC</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1.25</v>
+        <v>40000</v>
       </c>
       <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>mgr_salary</t>
+          <t>burden_uplift</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>140000</v>
+        <v>0.28</v>
       </c>
       <c r="C26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>physical_touch_share</t>
+          <t>lead_premium</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.35</v>
+        <v>1.25</v>
       </c>
       <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>day_one_reach</t>
+          <t>mgr_salary</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.55</v>
+        <v>140000</v>
       </c>
       <c r="C28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>reach_decay_exponent</t>
+          <t>physical_touch_share</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.6</v>
+        <v>0.35</v>
       </c>
       <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>parts_shipment_share</t>
+          <t>day_one_reach</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1378,464 +1095,918 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>cost_per_shipment</t>
+          <t>reach_decay_exponent</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>38</v>
+        <v>0.6</v>
       </c>
       <c r="C31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>depots_per_campus_share</t>
+          <t>parts_shipment_share</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>0.64</v>
+        <v>0.55</v>
       </c>
       <c r="C32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>depot_fixed_cost</t>
+          <t>cost_per_shipment</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>60000</v>
+        <v>38</v>
       </c>
       <c r="C33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>depot_variable_per_shipment</t>
+          <t>depots_per_campus_share</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>6</v>
+        <v>0.64</v>
       </c>
       <c r="C34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>stock_value_per_campus</t>
+          <t>depot_fixed_cost</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>45000</v>
+        <v>60000</v>
       </c>
       <c r="C35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>stock_carrying_cost</t>
+          <t>depot_variable_per_shipment</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0.18</v>
+        <v>6</v>
       </c>
       <c r="C36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>smart_hands_dispatch_cost</t>
+          <t>stock_value_per_campus</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>165</v>
+        <v>45000</v>
       </c>
       <c r="C37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>oem_attach_share</t>
+          <t>stock_carrying_cost</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>0.45</v>
+        <v>0.18</v>
       </c>
       <c r="C38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>oem_cost_per_incident</t>
+          <t>smart_hands_dispatch_cost</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>55</v>
+        <v>165</v>
       </c>
       <c r="C39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>break_fix_share</t>
+          <t>oem_attach_share</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>0.6</v>
+        <v>0.45</v>
       </c>
       <c r="C40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>devices_per_user</t>
+          <t>oem_cost_per_incident</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1.2</v>
+        <v>55</v>
       </c>
       <c r="C41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>refresh_cycle_years</t>
+          <t>break_fix_share</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>4</v>
+        <v>0.6</v>
       </c>
       <c r="C42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>zero_touch_ceiling</t>
+          <t>devices_per_user</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.85</v>
+        <v>1.2</v>
       </c>
       <c r="C43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>refresh_touch_cost</t>
+          <t>refresh_cycle_years</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>95</v>
+        <v>4</v>
       </c>
       <c r="C44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>refresh_shipping_cost</t>
+          <t>zero_touch_ceiling</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>24</v>
+        <v>0.85</v>
       </c>
       <c r="C45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>current_field_techs</t>
+          <t>refresh_touch_cost</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>150</v>
+        <v>95</v>
       </c>
       <c r="C46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>current_mgmt_overhead</t>
+          <t>refresh_shipping_cost</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>0.16</v>
+        <v>24</v>
       </c>
       <c r="C47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>current_logistics_spend</t>
+          <t>current_field_techs</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>900000</v>
+        <v>150</v>
       </c>
       <c r="C48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>severance_per_exit</t>
+          <t>current_mgmt_overhead</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>30000</v>
+        <v>0.16</v>
       </c>
       <c r="C49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>hire_train_per_add</t>
+          <t>current_logistics_spend</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>12000</v>
+        <v>900000</v>
       </c>
       <c r="C50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>parallel_run_months</t>
+          <t>severance_per_exit</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>2</v>
+        <v>30000</v>
       </c>
       <c r="C51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>program_mgmt_per_step</t>
+          <t>hire_train_per_add</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>150000</v>
+        <v>12000</v>
       </c>
       <c r="C52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>wage_escalation</t>
+          <t>parallel_run_months</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0.03</v>
+        <v>2</v>
       </c>
       <c r="C53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>discount_rate</t>
+          <t>program_mgmt_per_step</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>0.08</v>
+        <v>150000</v>
       </c>
       <c r="C54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>attrition_rate</t>
+          <t>wage_escalation</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>0.15</v>
+        <v>0.03</v>
       </c>
       <c r="C55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>step_year_ramp</t>
+          <t>discount_rate</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>0.6</v>
+        <v>0.08</v>
       </c>
       <c r="C56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>dispatch_rate_incident_remote</t>
+          <t>attrition_rate</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="C57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>dispatch_rate_request_remote</t>
+          <t>step_year_ramp</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>0.35</v>
+        <v>0.6</v>
       </c>
       <c r="C58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>shipment_rate_incident</t>
+          <t>dispatch_rate_incident_remote</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.18</v>
+        <v>0.12</v>
       </c>
       <c r="C59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>shipment_rate_request</t>
+          <t>dispatch_rate_request_remote</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
       <c r="C60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>dispatch_cost_NAM</t>
+          <t>shipment_rate_incident</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>375</v>
+        <v>0.18</v>
       </c>
       <c r="C61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>dispatch_cost_LATAM</t>
+          <t>shipment_rate_request</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>185</v>
+        <v>0.45</v>
       </c>
       <c r="C62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>dispatch_cost_EMEA</t>
+          <t>dispatch_cost_NAM</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>325</v>
+        <v>375</v>
       </c>
       <c r="C63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>dispatch_cost_APJC</t>
+          <t>dispatch_cost_LATAM</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>165</v>
+        <v>185</v>
       </c>
       <c r="C64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>shipment_cost_NAM</t>
+          <t>dispatch_cost_EMEA</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>55</v>
+        <v>325</v>
       </c>
       <c r="C65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>shipment_cost_LATAM</t>
+          <t>dispatch_cost_APJC</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>75</v>
+        <v>165</v>
       </c>
       <c r="C66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>shipment_cost_EMEA</t>
+          <t>shipment_cost_NAM</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>shipment_cost_APJC</t>
+          <t>shipment_cost_LATAM</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="C68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>overlay_virtual_techs</t>
+          <t>shipment_cost_EMEA</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="C69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>overlay_depot_techs_per_depot_campus</t>
+          <t>shipment_cost_APJC</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="C70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>overlay_tech_bar_threshold_users</t>
+          <t>overlay_virtual_techs</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>400</v>
+        <v>0</v>
       </c>
       <c r="C71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>staging_radius_miles</t>
+          <t>overlay_depot_techs_per_depot_campus</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="C72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>overlay_tech_bar_threshold_users</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>400</v>
+      </c>
+      <c r="C73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>quarantine_hold_days</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>14</v>
+      </c>
+      <c r="C74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>smart_hands_max_tot_minutes</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>60</v>
+      </c>
+      <c r="C75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ratio_guardrail_seats_per_tech</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>600</v>
+      </c>
+      <c r="C76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>working_days_month</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>22</v>
+      </c>
+      <c r="C77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>fmo_tickets_per_tech_day</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>7</v>
+      </c>
+      <c r="C78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>role_lanes</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>["Desktop-Incident", "Desktop-Requests", "Remote-Desktop", "Staging", "Site-Lead", "Telecom", "Network-VDI", "Projects"]</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>role_lane_primary_mix</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>{"Desktop-Incident": 0.35, "Desktop-Requests": 0.3, "Remote-Desktop": 0.15, "Staging": 0.05, "Site-Lead": 0.05, "Telecom": 0.04, "Network-VDI": 0.03, "Projects": 0.03}</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>role_lane_secondary_default</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Desktop-Requests</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>role_lane_tertiary_default</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Projects</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>schedule_lanes</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>["M", "TL", "T", "W", "S", "RR"]</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>vac_sick_uplift</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="C84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>travel_utilization</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>sla_mix_2h</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>sla_mix_4h</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>sla_mix_nbd</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>sla_mix_extended_hours</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>sla_uplift_2h</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>sla_uplift_4h</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="C91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>sla_uplift_nbd</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>0</v>
+      </c>
+      <c r="C92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>sla_uplift_extended_hours</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="C93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>critical_24x7_floor_techs</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>2</v>
+      </c>
+      <c r="C94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>vc_validation_load_factor</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="C95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>badged_share</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="C96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>partner_remote_share</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>on_call_enabled</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>0</v>
+      </c>
+      <c r="C98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>on_call_cost_per_tech_day</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>85</v>
+      </c>
+      <c r="C99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>fail_rate_desktop</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="C100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>fail_rate_laptop</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>use_fail_rate_bootstrap</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>0</v>
+      </c>
+      <c r="C102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>time_on_task_minutes_default</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>45</v>
+      </c>
+      <c r="C103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>volume_change_band</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>cost_validity_days</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>90</v>
+      </c>
+      <c r="C105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>warranty_labor_credit_per_event</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>0</v>
+      </c>
+      <c r="C106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>oppm_hourly_multiplier</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>hours_per_year_tm</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>2080</v>
+      </c>
+      <c r="C108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>sla_dispatch_urgency</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="C109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>fast_sla_spares_flag</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>1</v>
+      </c>
+      <c r="C110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>rate_note</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Modern placeholders only. Reference Deals G–I inform structure; do not ship 2012 wage/unit tables.</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>catchment_note</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Local if haversine miles ≤ staging_radius_miles (25) OR estimated drive minutes ≤ drive_minutes (60) at avg_drive_speed_mph (40 → ~40 mi for the 1-hr limb; engine uses the more inclusive bound). Remote+dispatch only when tpd &lt; remote_max_tpd (1.2) and outside local range; otherwise far sites promote to Staffed. drive_radius_km is legacy/unused.</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>